<commit_message>
Fix Generator group id in import file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DqqL6EB7PmiWrNzo7cqUca
</commit_message>
<xml_diff>
--- a/imports/gen_2026-10-29_generator.xlsx
+++ b/imports/gen_2026-10-29_generator.xlsx
@@ -1113,11 +1113,11 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
@@ -1471,11 +1471,11 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -1839,11 +1839,11 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -2172,11 +2172,11 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -2550,11 +2550,11 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -2858,11 +2858,11 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -3199,11 +3199,11 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
@@ -3517,11 +3517,11 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -3908,11 +3908,11 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4193,11 +4193,11 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>154216285</v>
+        <v>155938256</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Генераторы</t>
+          <t>Генератори</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">

</xml_diff>